<commit_message>
Complete Stage 4: Add PNJ Technical Specification, update prompt log and Excel cover
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-12-pnj-financials.xlsx
+++ b/models/builds/2026-05-12-pnj-financials.xlsx
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="322">
   <si>
     <t>UNIVERSITY OF HAWAIʻI AT MĀNOA · SHIDLER COLLEGE OF BUSINESS</t>
   </si>
@@ -974,43 +974,43 @@
     <t>Company</t>
   </si>
   <si>
-    <t>[Your Company Name]</t>
+    <t>Phu Nhuan Jewelry JSC (PNJ)</t>
   </si>
   <si>
     <t>Ticker</t>
   </si>
   <si>
-    <t>[TICKER]</t>
+    <t>PNJ</t>
   </si>
   <si>
     <t>Industry</t>
   </si>
   <si>
-    <t>[Industry]</t>
+    <t>Retail/Jewelry</t>
   </si>
   <si>
     <t>Fiscal Year (current)</t>
   </si>
   <si>
-    <t>[FYYYYY]</t>
-  </si>
-  <si>
     <t>Fiscal Year (prior)</t>
   </si>
   <si>
     <t>Data Source</t>
   </si>
   <si>
-    <t>[SEC EDGAR 10-K URL / Yahoo Finance / etc.]</t>
+    <t>https://dstock.vndirect.com.vn</t>
   </si>
   <si>
     <t>Units</t>
   </si>
   <si>
+    <t>All figures in Billion VND</t>
+  </si>
+  <si>
     <t>Tax Rate</t>
   </si>
   <si>
-    <t>[Statutory 21% / Effective rate from financials — and why]</t>
+    <t>20% (Standard VN Corporate Tax)</t>
   </si>
   <si>
     <t>Cost of Capital</t>
@@ -3436,32 +3436,32 @@
       <c r="B7" s="50" t="s">
         <v>293</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>294</v>
+      <c r="C7" s="8">
+        <v>2025</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="50" t="s">
-        <v>295</v>
-      </c>
-      <c r="C8" s="8" t="s">
         <v>294</v>
+      </c>
+      <c r="C8" s="8">
+        <v>2024</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="50" t="s">
+        <v>295</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>296</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="50" t="s">
+        <v>297</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>298</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">

</xml_diff>